<commit_message>
Actualizando la metadata y modificando el mensaje de error con el estado
</commit_message>
<xml_diff>
--- a/metadata/metadata_estadisticas_FP.xlsx
+++ b/metadata/metadata_estadisticas_FP.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/djurado/Projects/FP-History/metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82BFC8A1-A491-0A46-8676-8AE0C96663D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{346892F9-0972-194A-84F4-490FF95409EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1640" yWindow="780" windowWidth="29400" windowHeight="18460" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TPL_2022_2" sheetId="13" r:id="rId1"/>
@@ -18,8 +18,10 @@
     <sheet name="TPL_2023_2" sheetId="12" r:id="rId3"/>
     <sheet name="TPL_2024_1" sheetId="10" r:id="rId4"/>
     <sheet name="TPL_2024_2" sheetId="7" r:id="rId5"/>
-    <sheet name="TPL_2025_1" sheetId="8" r:id="rId6"/>
-    <sheet name="TPL_2025_2" sheetId="9" r:id="rId7"/>
+    <sheet name="TPL_2025_0" sheetId="15" r:id="rId6"/>
+    <sheet name="TPL_2025_1" sheetId="8" r:id="rId7"/>
+    <sheet name="TPL_2025_2" sheetId="9" r:id="rId8"/>
+    <sheet name="TPL_2026_0" sheetId="17" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="68">
   <si>
     <t/>
   </si>
@@ -238,6 +240,12 @@
   <si>
     <t>Numpy</t>
   </si>
+  <si>
+    <t>REVISADO_X_ESTUDIANTE</t>
+  </si>
+  <si>
+    <t>Lógica</t>
+  </si>
 </sst>
 </file>
 
@@ -384,7 +392,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -421,11 +429,644 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="99">
+  <dxfs count="150">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color indexed="65"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4472C4"/>
+          <bgColor rgb="FF4472C4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color indexed="65"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4472C4"/>
+          <bgColor rgb="FF4472C4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color indexed="65"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4472C4"/>
+          <bgColor rgb="FF4472C4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color indexed="65"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4472C4"/>
+          <bgColor rgb="FF4472C4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color indexed="65"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4472C4"/>
+          <bgColor rgb="FF4472C4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color indexed="65"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4472C4"/>
+          <bgColor rgb="FF4472C4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color indexed="65"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4472C4"/>
+          <bgColor rgb="FF4472C4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -627,7 +1268,7 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color indexed="65"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="none"/>
@@ -652,35 +1293,98 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color indexed="65"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF4472C4"/>
           <bgColor rgb="FF4472C4"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color indexed="65"/>
       </font>
       <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
@@ -689,35 +1393,38 @@
           <bgColor rgb="FF4472C4"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color indexed="65"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF4472C4"/>
           <bgColor rgb="FF4472C4"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FFFFFFFF"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color indexed="65"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
       </font>
       <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
@@ -731,7 +1438,19 @@
     <dxf>
       <font>
         <b/>
-        <color rgb="FFFFFFFF"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color indexed="65"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
       </font>
       <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
@@ -754,7 +1473,7 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color indexed="65"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="none"/>
@@ -780,7 +1499,7 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color indexed="65"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="none"/>
@@ -806,7 +1525,7 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color indexed="65"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="none"/>
@@ -832,12 +1551,11 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+        <color indexed="65"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF4472C4"/>
@@ -858,6 +1576,272 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="0"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
         <color rgb="FFFFFFFF"/>
         <name val="Calibri"/>
         <family val="2"/>
@@ -888,13 +1872,13 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF4472C4"/>
           <bgColor rgb="FF4472C4"/>
         </patternFill>
       </fill>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -938,31 +1922,17 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF4472C4"/>
           <bgColor rgb="FF4472C4"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
         <color rgb="FFFFFFFF"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
       </font>
       <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
@@ -971,24 +1941,12 @@
           <bgColor rgb="FF4472C4"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
         <color rgb="FFFFFFFF"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
       </font>
       <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
@@ -997,7 +1955,7 @@
           <bgColor rgb="FF4472C4"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1016,12 +1974,14 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF4472C4"/>
           <bgColor rgb="FF4472C4"/>
         </patternFill>
       </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1040,6 +2000,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF4472C4"/>
@@ -1072,11 +2033,24 @@
           <bgColor rgb="FF4472C4"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
         <color rgb="FFFFFFFF"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
       </font>
       <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
@@ -1085,7 +2059,7 @@
           <bgColor rgb="FF4472C4"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1104,13 +2078,13 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF4472C4"/>
           <bgColor rgb="FF4472C4"/>
         </patternFill>
       </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1129,13 +2103,13 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF4472C4"/>
           <bgColor rgb="FF4472C4"/>
         </patternFill>
       </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1174,6 +2148,247 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4472C4"/>
+          <bgColor rgb="FF4472C4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4472C4"/>
+          <bgColor rgb="FF4472C4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4472C4"/>
+          <bgColor rgb="FF4472C4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4472C4"/>
+          <bgColor rgb="FF4472C4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4472C4"/>
+          <bgColor rgb="FF4472C4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4472C4"/>
+          <bgColor rgb="FF4472C4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4472C4"/>
+          <bgColor rgb="FF4472C4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4472C4"/>
+          <bgColor rgb="FF4472C4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4472C4"/>
+          <bgColor rgb="FF4472C4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4472C4"/>
+          <bgColor rgb="FF4472C4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
         <color indexed="65"/>
         <name val="Calibri"/>
         <family val="2"/>
@@ -1978,6 +3193,7 @@
           <bgColor theme="4"/>
         </patternFill>
       </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -2021,7 +3237,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="1" formatCode="0"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor theme="4"/>
@@ -2041,6 +3257,56 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
         <color indexed="65"/>
         <name val="Calibri"/>
         <family val="2"/>
@@ -2057,7 +3323,19 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
         <color indexed="65"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
       </font>
       <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
@@ -2071,7 +3349,19 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
         <color indexed="65"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
       </font>
       <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
@@ -2177,7 +3467,6 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF4472C4"/>
@@ -2198,57 +3487,6 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color indexed="65"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF4472C4"/>
-          <bgColor rgb="FF4472C4"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color indexed="65"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF4472C4"/>
-          <bgColor rgb="FF4472C4"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
         <color theme="0"/>
         <name val="Calibri"/>
         <family val="2"/>
@@ -2279,14 +3517,13 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor theme="4"/>
           <bgColor theme="4"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -2312,7 +3549,6 @@
           <bgColor theme="4"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -2338,7 +3574,6 @@
           <bgColor theme="4"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -2382,6 +3617,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor theme="4"/>
@@ -2406,27 +3642,87 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor theme="4"/>
           <bgColor theme="4"/>
         </patternFill>
       </fill>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
         <color theme="0"/>
-      </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor theme="4"/>
           <bgColor theme="4"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -2526,37 +3822,37 @@
     <tableColumn id="4" xr3:uid="{36EE22E4-B443-794A-AF38-7209D9285AAB}" name="SIT"/>
     <tableColumn id="5" xr3:uid="{491FD25F-711A-0E48-AF14-B323B23C7F48}" name="PARCIAL"/>
     <tableColumn id="6" xr3:uid="{9254419B-9CAC-3248-8409-9F3DA0AB8120}" name="EXAMEN 1E"/>
-    <tableColumn id="7" xr3:uid="{E2351D4B-BF02-B844-8515-4D6B156C4343}" name="TEMA 1E-1" dataDxfId="74"/>
-    <tableColumn id="8" xr3:uid="{4D1AE9CA-AD56-1344-9D58-C34FB41C2804}" name="TEMA 1E-2" dataDxfId="73"/>
-    <tableColumn id="9" xr3:uid="{2FF825E5-706C-B640-A6FB-303A9777FBDE}" name="TEMA 1E-3" dataDxfId="72"/>
-    <tableColumn id="33" xr3:uid="{0112D43B-0180-C54F-96CC-485AED172C51}" name="TEMA 1E-4" dataDxfId="71"/>
-    <tableColumn id="10" xr3:uid="{D2AB48DC-2AE1-CF4B-8E83-C264489CFBDE}" name="TEMA 1E-5" dataDxfId="70"/>
-    <tableColumn id="12" xr3:uid="{60ADCE4B-4C66-884E-A320-9BD78CC0989E}" name="ESTADO 1E" dataDxfId="69"/>
-    <tableColumn id="13" xr3:uid="{D197CEF1-1F66-764B-9BD4-D1790CE662B9}" name="FINAL" dataDxfId="68"/>
-    <tableColumn id="14" xr3:uid="{885E880D-026D-9044-BAB1-1889D6096980}" name="EXAMEN 2E" dataDxfId="67"/>
-    <tableColumn id="15" xr3:uid="{4E5FD8BB-05F5-C342-A577-C7EAC9385C6E}" name="TEMA 2E-1.1" dataDxfId="66"/>
-    <tableColumn id="16" xr3:uid="{D01919E8-8EC2-F741-8D03-6D550364E9D9}" name="TEMA 2E-1.2" dataDxfId="65"/>
-    <tableColumn id="18" xr3:uid="{0F7B5770-0B84-7542-A668-99EC8C28A3CA}" name="TEMA 2E-1.3" dataDxfId="64"/>
-    <tableColumn id="20" xr3:uid="{D3300D6A-D0CE-474F-BADA-E37A7ED0F79D}" name="TEMA 2E-1.4" dataDxfId="63"/>
-    <tableColumn id="21" xr3:uid="{DEC1B0EF-05BA-DD41-8D60-04F2E35CEF06}" name="TEMA 2E-1.5" dataDxfId="62"/>
-    <tableColumn id="22" xr3:uid="{1C5C625D-1D92-D04A-A7D0-F39D9645A11C}" name="TEMA 2E-1.6" dataDxfId="61"/>
-    <tableColumn id="23" xr3:uid="{53242850-8D10-3747-BD5A-223925789073}" name="TEMA 2E-2.1" dataDxfId="60"/>
-    <tableColumn id="24" xr3:uid="{E7E0E6E5-F05C-7B40-A20F-2BFAAE8AE215}" name="TEMA 2E-2.2" dataDxfId="59"/>
-    <tableColumn id="25" xr3:uid="{9CA7EFA7-AB6A-5B48-808C-99065509CCDF}" name="TEMA 2E-2.3" dataDxfId="58"/>
-    <tableColumn id="34" xr3:uid="{FF2E526D-4375-B44A-A888-CEBB555A9531}" name="TEMA 2E-BONO" dataDxfId="57"/>
-    <tableColumn id="35" xr3:uid="{0D9CC297-0CF6-5E48-B539-C8E821A626A8}" name="ESTADO 2E" dataDxfId="56"/>
-    <tableColumn id="26" xr3:uid="{D79DC385-3CF2-9D44-9CCF-39B5115AE804}" name="MEJORAMIENTO" dataDxfId="55"/>
-    <tableColumn id="28" xr3:uid="{A6A3E644-D474-604F-A2FD-0EB3A41B2810}" name="EXAMEN 3E" dataDxfId="54"/>
-    <tableColumn id="29" xr3:uid="{AA7DFEBE-99A4-D447-8DAB-2861E78F86E7}" name="TEMA 3E-1" dataDxfId="53"/>
-    <tableColumn id="30" xr3:uid="{08751A4D-AE15-3F41-A1E5-5E169DBE6EB6}" name="TEMA 3E-2" dataDxfId="52"/>
-    <tableColumn id="32" xr3:uid="{053CC1C6-8559-B540-9E4D-FDFCDD6B3B97}" name="TEMA 3E-3" dataDxfId="51"/>
-    <tableColumn id="36" xr3:uid="{7EA65E44-1BBE-E144-9453-97EAD558B1D1}" name="TEMA 3E-4" dataDxfId="50"/>
-    <tableColumn id="37" xr3:uid="{AC5D6180-9071-2D4D-B1A4-0D9908969184}" name="TEMA 3E-5" dataDxfId="49"/>
-    <tableColumn id="38" xr3:uid="{643C15FA-AB6F-F342-9EAC-CD619414C47C}" name="ESTADO 3E" dataDxfId="48"/>
-    <tableColumn id="39" xr3:uid="{C283C9B3-E8D9-C243-9340-82888F8ACCDD}" name="PRACTICO" dataDxfId="47"/>
-    <tableColumn id="40" xr3:uid="{FA4BB7E0-1D8F-4949-BD6C-A99D7672A2AC}" name="TALLERES" dataDxfId="46"/>
-    <tableColumn id="41" xr3:uid="{D0BF6A30-E29B-BB40-92E1-B9ABFAC4FD07}" name="PARTICIPACION" dataDxfId="45"/>
-    <tableColumn id="42" xr3:uid="{641F4CCE-AA19-E244-B55C-010DE32B5E0B}" name="ESTADO" dataDxfId="44"/>
+    <tableColumn id="7" xr3:uid="{E2351D4B-BF02-B844-8515-4D6B156C4343}" name="TEMA 1E-1" dataDxfId="123"/>
+    <tableColumn id="8" xr3:uid="{4D1AE9CA-AD56-1344-9D58-C34FB41C2804}" name="TEMA 1E-2" dataDxfId="122"/>
+    <tableColumn id="9" xr3:uid="{2FF825E5-706C-B640-A6FB-303A9777FBDE}" name="TEMA 1E-3" dataDxfId="121"/>
+    <tableColumn id="33" xr3:uid="{0112D43B-0180-C54F-96CC-485AED172C51}" name="TEMA 1E-4" dataDxfId="120"/>
+    <tableColumn id="10" xr3:uid="{D2AB48DC-2AE1-CF4B-8E83-C264489CFBDE}" name="TEMA 1E-5" dataDxfId="119"/>
+    <tableColumn id="12" xr3:uid="{60ADCE4B-4C66-884E-A320-9BD78CC0989E}" name="ESTADO 1E" dataDxfId="118"/>
+    <tableColumn id="13" xr3:uid="{D197CEF1-1F66-764B-9BD4-D1790CE662B9}" name="FINAL" dataDxfId="117"/>
+    <tableColumn id="14" xr3:uid="{885E880D-026D-9044-BAB1-1889D6096980}" name="EXAMEN 2E" dataDxfId="116"/>
+    <tableColumn id="15" xr3:uid="{4E5FD8BB-05F5-C342-A577-C7EAC9385C6E}" name="TEMA 2E-1.1" dataDxfId="115"/>
+    <tableColumn id="16" xr3:uid="{D01919E8-8EC2-F741-8D03-6D550364E9D9}" name="TEMA 2E-1.2" dataDxfId="114"/>
+    <tableColumn id="18" xr3:uid="{0F7B5770-0B84-7542-A668-99EC8C28A3CA}" name="TEMA 2E-1.3" dataDxfId="113"/>
+    <tableColumn id="20" xr3:uid="{D3300D6A-D0CE-474F-BADA-E37A7ED0F79D}" name="TEMA 2E-1.4" dataDxfId="112"/>
+    <tableColumn id="21" xr3:uid="{DEC1B0EF-05BA-DD41-8D60-04F2E35CEF06}" name="TEMA 2E-1.5" dataDxfId="111"/>
+    <tableColumn id="22" xr3:uid="{1C5C625D-1D92-D04A-A7D0-F39D9645A11C}" name="TEMA 2E-1.6" dataDxfId="110"/>
+    <tableColumn id="23" xr3:uid="{53242850-8D10-3747-BD5A-223925789073}" name="TEMA 2E-2.1" dataDxfId="109"/>
+    <tableColumn id="24" xr3:uid="{E7E0E6E5-F05C-7B40-A20F-2BFAAE8AE215}" name="TEMA 2E-2.2" dataDxfId="108"/>
+    <tableColumn id="25" xr3:uid="{9CA7EFA7-AB6A-5B48-808C-99065509CCDF}" name="TEMA 2E-2.3" dataDxfId="107"/>
+    <tableColumn id="34" xr3:uid="{FF2E526D-4375-B44A-A888-CEBB555A9531}" name="TEMA 2E-BONO" dataDxfId="106"/>
+    <tableColumn id="35" xr3:uid="{0D9CC297-0CF6-5E48-B539-C8E821A626A8}" name="ESTADO 2E" dataDxfId="105"/>
+    <tableColumn id="26" xr3:uid="{D79DC385-3CF2-9D44-9CCF-39B5115AE804}" name="MEJORAMIENTO" dataDxfId="104"/>
+    <tableColumn id="28" xr3:uid="{A6A3E644-D474-604F-A2FD-0EB3A41B2810}" name="EXAMEN 3E" dataDxfId="103"/>
+    <tableColumn id="29" xr3:uid="{AA7DFEBE-99A4-D447-8DAB-2861E78F86E7}" name="TEMA 3E-1" dataDxfId="102"/>
+    <tableColumn id="30" xr3:uid="{08751A4D-AE15-3F41-A1E5-5E169DBE6EB6}" name="TEMA 3E-2" dataDxfId="101"/>
+    <tableColumn id="32" xr3:uid="{053CC1C6-8559-B540-9E4D-FDFCDD6B3B97}" name="TEMA 3E-3" dataDxfId="100"/>
+    <tableColumn id="36" xr3:uid="{7EA65E44-1BBE-E144-9453-97EAD558B1D1}" name="TEMA 3E-4" dataDxfId="99"/>
+    <tableColumn id="37" xr3:uid="{AC5D6180-9071-2D4D-B1A4-0D9908969184}" name="TEMA 3E-5" dataDxfId="98"/>
+    <tableColumn id="38" xr3:uid="{643C15FA-AB6F-F342-9EAC-CD619414C47C}" name="ESTADO 3E" dataDxfId="97"/>
+    <tableColumn id="39" xr3:uid="{C283C9B3-E8D9-C243-9340-82888F8ACCDD}" name="PRACTICO" dataDxfId="96"/>
+    <tableColumn id="40" xr3:uid="{FA4BB7E0-1D8F-4949-BD6C-A99D7672A2AC}" name="TALLERES" dataDxfId="95"/>
+    <tableColumn id="41" xr3:uid="{D0BF6A30-E29B-BB40-92E1-B9ABFAC4FD07}" name="PARTICIPACION" dataDxfId="94"/>
+    <tableColumn id="42" xr3:uid="{641F4CCE-AA19-E244-B55C-010DE32B5E0B}" name="ESTADO" dataDxfId="93"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -2572,29 +3868,29 @@
     <tableColumn id="4" xr3:uid="{105F4267-2BD8-D94B-99AD-D6D582F11E0B}" name="SIT"/>
     <tableColumn id="5" xr3:uid="{ABD75318-A9F8-5442-A72E-80585A97D3E3}" name="PARCIAL"/>
     <tableColumn id="6" xr3:uid="{5DBBE1E6-2958-A048-AB64-54C7A4773152}" name="EXAMEN 1E"/>
-    <tableColumn id="7" xr3:uid="{79E54B85-E1EA-0245-AD3A-1F32E12BA32B}" name="TEMA 1E-1" dataDxfId="43"/>
-    <tableColumn id="8" xr3:uid="{026EACC3-BAF7-5F4F-A411-F519F374B5FE}" name="TEMA 1E-2" dataDxfId="42"/>
-    <tableColumn id="9" xr3:uid="{D3F13721-0521-4041-AC70-77CEA05CF1F0}" name="TEMA 1E-3" dataDxfId="41"/>
-    <tableColumn id="33" xr3:uid="{712C19D8-0A2E-2948-A2B1-C761B135A2DE}" name="TEMA 1E-4" dataDxfId="40"/>
-    <tableColumn id="10" xr3:uid="{D8F1D1AD-4859-0242-A860-9473E1D1625B}" name="TEMA 1E-5" dataDxfId="39"/>
-    <tableColumn id="12" xr3:uid="{2AF5F57F-87E7-3F49-8B79-F002C578B08F}" name="ESTADO 1E" dataDxfId="38"/>
-    <tableColumn id="13" xr3:uid="{209F8CBB-55C7-C04E-ACF7-B40E26E32273}" name="FINAL" dataDxfId="37"/>
-    <tableColumn id="14" xr3:uid="{B21CCBC6-B090-A849-AC73-E2C27B1BA9E4}" name="EXAMEN 2E" dataDxfId="36"/>
-    <tableColumn id="15" xr3:uid="{F795D6BD-C3F9-3548-9DAF-14AB85C15F3F}" name="TEMA 2E-1.1" dataDxfId="35"/>
-    <tableColumn id="16" xr3:uid="{A3C23799-56F2-7B45-9542-C6D943DD3E27}" name="TEMA 2E-1.2" dataDxfId="34"/>
-    <tableColumn id="18" xr3:uid="{E81A55ED-0575-8D4F-97B6-36B8F28821F8}" name="TEMA 2E-2" dataDxfId="33"/>
-    <tableColumn id="20" xr3:uid="{A6B9FC36-6D10-6847-852C-79B4FE80307B}" name="ESTADO 2E" dataDxfId="32"/>
-    <tableColumn id="21" xr3:uid="{82011D67-6871-544A-9178-FA326DCFB453}" name="MEJORAMIENTO" dataDxfId="31"/>
-    <tableColumn id="22" xr3:uid="{EDCDC284-1C63-8845-8BE3-DDC80852BA86}" name="EXAMEN 3E" dataDxfId="30"/>
-    <tableColumn id="23" xr3:uid="{42627284-0C57-134E-973A-B8BEC0469BA5}" name="TEMA 3E-1" dataDxfId="29"/>
-    <tableColumn id="24" xr3:uid="{42215CC0-B24E-BD4D-837E-20EEA74036AD}" name="TEMA 3E-2" dataDxfId="28"/>
-    <tableColumn id="25" xr3:uid="{BE55CDCB-B2BE-A049-9ED6-476C018D7264}" name="TEMA 3E-3" dataDxfId="27"/>
-    <tableColumn id="34" xr3:uid="{E101B822-E8AA-C549-B101-4F346D976001}" name="TEMA 3E-4" dataDxfId="26"/>
-    <tableColumn id="35" xr3:uid="{1578CDC8-17F2-524A-8D98-3143C028FE55}" name="ESTADO 3E" dataDxfId="25"/>
-    <tableColumn id="26" xr3:uid="{C4479F82-400A-274D-982F-56EE1C7278C7}" name="PRACTICO" dataDxfId="24"/>
-    <tableColumn id="28" xr3:uid="{5C3A5E06-2C3A-1F45-A0D2-8DB9BDD43078}" name="TALLERES" dataDxfId="23"/>
-    <tableColumn id="29" xr3:uid="{ADFE90B3-0E29-E940-A344-2F1530105E94}" name="PARTICIPACION" dataDxfId="22"/>
-    <tableColumn id="30" xr3:uid="{7698038C-00CC-FD43-897B-65B1B038B1C1}" name="ESTADO" dataDxfId="21"/>
+    <tableColumn id="7" xr3:uid="{79E54B85-E1EA-0245-AD3A-1F32E12BA32B}" name="TEMA 1E-1" dataDxfId="92"/>
+    <tableColumn id="8" xr3:uid="{026EACC3-BAF7-5F4F-A411-F519F374B5FE}" name="TEMA 1E-2" dataDxfId="91"/>
+    <tableColumn id="9" xr3:uid="{D3F13721-0521-4041-AC70-77CEA05CF1F0}" name="TEMA 1E-3" dataDxfId="90"/>
+    <tableColumn id="33" xr3:uid="{712C19D8-0A2E-2948-A2B1-C761B135A2DE}" name="TEMA 1E-4" dataDxfId="89"/>
+    <tableColumn id="10" xr3:uid="{D8F1D1AD-4859-0242-A860-9473E1D1625B}" name="TEMA 1E-5" dataDxfId="88"/>
+    <tableColumn id="12" xr3:uid="{2AF5F57F-87E7-3F49-8B79-F002C578B08F}" name="ESTADO 1E" dataDxfId="87"/>
+    <tableColumn id="13" xr3:uid="{209F8CBB-55C7-C04E-ACF7-B40E26E32273}" name="FINAL" dataDxfId="86"/>
+    <tableColumn id="14" xr3:uid="{B21CCBC6-B090-A849-AC73-E2C27B1BA9E4}" name="EXAMEN 2E" dataDxfId="85"/>
+    <tableColumn id="15" xr3:uid="{F795D6BD-C3F9-3548-9DAF-14AB85C15F3F}" name="TEMA 2E-1.1" dataDxfId="84"/>
+    <tableColumn id="16" xr3:uid="{A3C23799-56F2-7B45-9542-C6D943DD3E27}" name="TEMA 2E-1.2" dataDxfId="83"/>
+    <tableColumn id="18" xr3:uid="{E81A55ED-0575-8D4F-97B6-36B8F28821F8}" name="TEMA 2E-2" dataDxfId="82"/>
+    <tableColumn id="20" xr3:uid="{A6B9FC36-6D10-6847-852C-79B4FE80307B}" name="ESTADO 2E" dataDxfId="81"/>
+    <tableColumn id="21" xr3:uid="{82011D67-6871-544A-9178-FA326DCFB453}" name="MEJORAMIENTO" dataDxfId="80"/>
+    <tableColumn id="22" xr3:uid="{EDCDC284-1C63-8845-8BE3-DDC80852BA86}" name="EXAMEN 3E" dataDxfId="79"/>
+    <tableColumn id="23" xr3:uid="{42627284-0C57-134E-973A-B8BEC0469BA5}" name="TEMA 3E-1" dataDxfId="78"/>
+    <tableColumn id="24" xr3:uid="{42215CC0-B24E-BD4D-837E-20EEA74036AD}" name="TEMA 3E-2" dataDxfId="77"/>
+    <tableColumn id="25" xr3:uid="{BE55CDCB-B2BE-A049-9ED6-476C018D7264}" name="TEMA 3E-3" dataDxfId="76"/>
+    <tableColumn id="34" xr3:uid="{E101B822-E8AA-C549-B101-4F346D976001}" name="TEMA 3E-4" dataDxfId="75"/>
+    <tableColumn id="35" xr3:uid="{1578CDC8-17F2-524A-8D98-3143C028FE55}" name="ESTADO 3E" dataDxfId="74"/>
+    <tableColumn id="26" xr3:uid="{C4479F82-400A-274D-982F-56EE1C7278C7}" name="PRACTICO" dataDxfId="73"/>
+    <tableColumn id="28" xr3:uid="{5C3A5E06-2C3A-1F45-A0D2-8DB9BDD43078}" name="TALLERES" dataDxfId="72"/>
+    <tableColumn id="29" xr3:uid="{ADFE90B3-0E29-E940-A344-2F1530105E94}" name="PARTICIPACION" dataDxfId="71"/>
+    <tableColumn id="30" xr3:uid="{7698038C-00CC-FD43-897B-65B1B038B1C1}" name="ESTADO" dataDxfId="70"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -2610,30 +3906,30 @@
     <tableColumn id="4" xr3:uid="{0AC9D01A-A923-F84C-AB65-93DF958A4AF4}" name="SIT"/>
     <tableColumn id="5" xr3:uid="{C355E8C4-4A2E-7F4F-8BEE-8D483CFCBA4C}" name="PARCIAL"/>
     <tableColumn id="6" xr3:uid="{23CECF01-E8A5-1948-AF70-4D43EECE2B07}" name="EXAMEN 1E"/>
-    <tableColumn id="7" xr3:uid="{F81C6692-FE02-2B4F-B6BE-E7F001B94F34}" name="TEMA 1E-1" dataDxfId="98"/>
-    <tableColumn id="8" xr3:uid="{171967B7-44EB-BF48-B4FF-EA4666E11E4B}" name="TEMA 1E-2" dataDxfId="97"/>
-    <tableColumn id="9" xr3:uid="{07A3232B-7DDE-7A4C-91FB-6D62B6413D04}" name="TEMA 1E-3" dataDxfId="96"/>
-    <tableColumn id="33" xr3:uid="{9E85CBA5-0B00-3D4D-BF0D-D76BCF271BD6}" name="TEMA 1E-4" dataDxfId="95"/>
-    <tableColumn id="10" xr3:uid="{84EF2217-8F86-E545-9E02-3AD4583F7EDA}" name="ESTADO 1E" dataDxfId="94"/>
-    <tableColumn id="12" xr3:uid="{0161A510-B91A-6F49-958C-6C66E4D63793}" name="FINAL" dataDxfId="93"/>
-    <tableColumn id="13" xr3:uid="{68879EE5-836B-2546-89C8-A3554B9A1660}" name="EXAMEN 2E" dataDxfId="92"/>
-    <tableColumn id="14" xr3:uid="{E3D3CCF1-F19D-644F-ABDD-065377D1C907}" name="TEMA 2E-1.1" dataDxfId="91"/>
-    <tableColumn id="15" xr3:uid="{01226A45-F178-9E4B-9E34-055CD1E517FC}" name="TEMA 2E-1.2" dataDxfId="90"/>
-    <tableColumn id="16" xr3:uid="{A3518E0B-5040-E941-AE58-C814A943B149}" name="TEMA 2E-2" dataDxfId="89"/>
-    <tableColumn id="18" xr3:uid="{05545699-A9E9-A040-9336-D0F2F8F85883}" name="ESTADO 2E" dataDxfId="88"/>
-    <tableColumn id="20" xr3:uid="{D8F1BA7D-2D5D-A243-82CF-781B8E8D50D2}" name="MEJORAMIENTO" dataDxfId="87"/>
-    <tableColumn id="21" xr3:uid="{01C3DF34-E48A-5A4C-83C4-27EFCBEDCC72}" name="EXAMEN 3E" dataDxfId="86"/>
-    <tableColumn id="22" xr3:uid="{20CAA21A-1904-2949-83F0-BFC8F897F1BF}" name="TEMA 3E-1.1" dataDxfId="85"/>
-    <tableColumn id="23" xr3:uid="{99C8B5C2-0AC2-BC42-8AF5-36F764EB3B1C}" name="TEMA 3E-1.2" dataDxfId="84"/>
-    <tableColumn id="24" xr3:uid="{401FD0F3-3D16-2945-864E-8253015942E7}" name="TEMA 3E-1.3" dataDxfId="83"/>
-    <tableColumn id="25" xr3:uid="{DB1E9C7F-DE7F-F743-940C-1C9B997A3F16}" name="TEMA 3E-2.1" dataDxfId="82"/>
-    <tableColumn id="34" xr3:uid="{B28854A0-53C2-F744-8C8B-DB10E6805ED5}" name="TEMA 3E-2.2" dataDxfId="81"/>
-    <tableColumn id="35" xr3:uid="{3B9FA228-5600-D141-8CA8-5EFC4925B4A0}" name="TEMA 3E-3" dataDxfId="80"/>
-    <tableColumn id="26" xr3:uid="{BB7FB6A7-D4A9-334E-B13E-F62B8F11C648}" name="ESTADO 3E" dataDxfId="79"/>
-    <tableColumn id="28" xr3:uid="{996A59EE-C748-2049-8D43-69A2E5783FA7}" name="PRACTICO" dataDxfId="78"/>
-    <tableColumn id="29" xr3:uid="{CDA3A075-E0E0-7946-BC28-ECFDE738E840}" name="TALLERES" dataDxfId="77"/>
-    <tableColumn id="30" xr3:uid="{8C12C22B-315D-AE44-83EB-43ED5B726BBA}" name="PARTICIPACION" dataDxfId="76"/>
-    <tableColumn id="32" xr3:uid="{DEA695EE-29CB-5043-A77F-38E1FB25C190}" name="ESTADO" dataDxfId="75"/>
+    <tableColumn id="7" xr3:uid="{F81C6692-FE02-2B4F-B6BE-E7F001B94F34}" name="TEMA 1E-1" dataDxfId="69"/>
+    <tableColumn id="8" xr3:uid="{171967B7-44EB-BF48-B4FF-EA4666E11E4B}" name="TEMA 1E-2" dataDxfId="68"/>
+    <tableColumn id="9" xr3:uid="{07A3232B-7DDE-7A4C-91FB-6D62B6413D04}" name="TEMA 1E-3" dataDxfId="67"/>
+    <tableColumn id="33" xr3:uid="{9E85CBA5-0B00-3D4D-BF0D-D76BCF271BD6}" name="TEMA 1E-4" dataDxfId="66"/>
+    <tableColumn id="10" xr3:uid="{84EF2217-8F86-E545-9E02-3AD4583F7EDA}" name="ESTADO 1E" dataDxfId="65"/>
+    <tableColumn id="12" xr3:uid="{0161A510-B91A-6F49-958C-6C66E4D63793}" name="FINAL" dataDxfId="64"/>
+    <tableColumn id="13" xr3:uid="{68879EE5-836B-2546-89C8-A3554B9A1660}" name="EXAMEN 2E" dataDxfId="63"/>
+    <tableColumn id="14" xr3:uid="{E3D3CCF1-F19D-644F-ABDD-065377D1C907}" name="TEMA 2E-1.1" dataDxfId="62"/>
+    <tableColumn id="15" xr3:uid="{01226A45-F178-9E4B-9E34-055CD1E517FC}" name="TEMA 2E-1.2" dataDxfId="61"/>
+    <tableColumn id="16" xr3:uid="{A3518E0B-5040-E941-AE58-C814A943B149}" name="TEMA 2E-2" dataDxfId="60"/>
+    <tableColumn id="18" xr3:uid="{05545699-A9E9-A040-9336-D0F2F8F85883}" name="ESTADO 2E" dataDxfId="59"/>
+    <tableColumn id="20" xr3:uid="{D8F1BA7D-2D5D-A243-82CF-781B8E8D50D2}" name="MEJORAMIENTO" dataDxfId="58"/>
+    <tableColumn id="21" xr3:uid="{01C3DF34-E48A-5A4C-83C4-27EFCBEDCC72}" name="EXAMEN 3E" dataDxfId="57"/>
+    <tableColumn id="22" xr3:uid="{20CAA21A-1904-2949-83F0-BFC8F897F1BF}" name="TEMA 3E-1.1" dataDxfId="56"/>
+    <tableColumn id="23" xr3:uid="{99C8B5C2-0AC2-BC42-8AF5-36F764EB3B1C}" name="TEMA 3E-1.2" dataDxfId="55"/>
+    <tableColumn id="24" xr3:uid="{401FD0F3-3D16-2945-864E-8253015942E7}" name="TEMA 3E-1.3" dataDxfId="54"/>
+    <tableColumn id="25" xr3:uid="{DB1E9C7F-DE7F-F743-940C-1C9B997A3F16}" name="TEMA 3E-2.1" dataDxfId="53"/>
+    <tableColumn id="34" xr3:uid="{B28854A0-53C2-F744-8C8B-DB10E6805ED5}" name="TEMA 3E-2.2" dataDxfId="52"/>
+    <tableColumn id="35" xr3:uid="{3B9FA228-5600-D141-8CA8-5EFC4925B4A0}" name="TEMA 3E-3" dataDxfId="51"/>
+    <tableColumn id="26" xr3:uid="{BB7FB6A7-D4A9-334E-B13E-F62B8F11C648}" name="ESTADO 3E" dataDxfId="50"/>
+    <tableColumn id="28" xr3:uid="{996A59EE-C748-2049-8D43-69A2E5783FA7}" name="PRACTICO" dataDxfId="49"/>
+    <tableColumn id="29" xr3:uid="{CDA3A075-E0E0-7946-BC28-ECFDE738E840}" name="TALLERES" dataDxfId="48"/>
+    <tableColumn id="30" xr3:uid="{8C12C22B-315D-AE44-83EB-43ED5B726BBA}" name="PARTICIPACION" dataDxfId="47"/>
+    <tableColumn id="32" xr3:uid="{DEA695EE-29CB-5043-A77F-38E1FB25C190}" name="ESTADO" dataDxfId="46"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -2649,27 +3945,27 @@
     <tableColumn id="4" xr3:uid="{72074798-5884-CF45-93B9-BFDB8FCA9620}" name="SIT"/>
     <tableColumn id="5" xr3:uid="{9A0886C4-1BB4-134B-BFED-D44FC2C8713E}" name="PARCIAL"/>
     <tableColumn id="6" xr3:uid="{FBB7EFBF-6CD4-454A-929B-2A25787A0C7A}" name="EXAMEN 1E"/>
-    <tableColumn id="7" xr3:uid="{7C47C583-6454-7143-9A5D-CA0D6855FA55}" name="TEMA 1E-1" dataDxfId="20"/>
-    <tableColumn id="8" xr3:uid="{A89283B0-5A62-E944-B1EC-A79C9E8F0E9C}" name="TEMA 1E-2" dataDxfId="19"/>
-    <tableColumn id="9" xr3:uid="{0DC7A31D-F4E5-774F-89FF-1A4E80909842}" name="TEMA 1E-3" dataDxfId="18"/>
-    <tableColumn id="33" xr3:uid="{DA4A822E-2817-1244-BA2A-953AAFCACBAF}" name="TEMA 1E-4" dataDxfId="17"/>
-    <tableColumn id="10" xr3:uid="{7466F1D5-8437-AC4A-980C-A5AE857FF3CC}" name="ESTADO 1E" dataDxfId="16"/>
-    <tableColumn id="12" xr3:uid="{05A41B80-085C-D543-BD2B-67ED67375527}" name="FINAL" dataDxfId="15"/>
-    <tableColumn id="13" xr3:uid="{D9FF644A-C9F5-BE41-9011-B7F715418CA3}" name="EXAMEN 2E" dataDxfId="14"/>
-    <tableColumn id="14" xr3:uid="{B3ACF5E8-6AF9-D34C-B79B-F7EE5D15BEB7}" name="TEMA 2E-1.1" dataDxfId="13"/>
-    <tableColumn id="15" xr3:uid="{C76E2C0D-F2A6-3845-9675-078249A7096C}" name="TEMA 2E-1.2" dataDxfId="12"/>
-    <tableColumn id="16" xr3:uid="{DAAB7757-1235-DB49-8EA1-58E9C72DDF81}" name="TEMA 2E-2" dataDxfId="11"/>
-    <tableColumn id="18" xr3:uid="{BB97EC96-F05F-8F4D-989A-F6B50584BDC6}" name="ESTADO 2E" dataDxfId="10"/>
-    <tableColumn id="20" xr3:uid="{63AED625-1A4B-E447-8861-521ED4352977}" name="MEJORAMIENTO" dataDxfId="9"/>
-    <tableColumn id="21" xr3:uid="{4BDB3BC1-0532-944E-871E-8263817D8B94}" name="EXAMEN 3E" dataDxfId="8"/>
-    <tableColumn id="22" xr3:uid="{CA5D9BF3-B8F4-9F4D-B6BA-5F14BCD7D396}" name="TEMA 3E-1" dataDxfId="7"/>
-    <tableColumn id="23" xr3:uid="{C7E4476F-7BB9-3043-BB4F-0470EB216E0F}" name="TEMA 3E-2" dataDxfId="6"/>
-    <tableColumn id="24" xr3:uid="{CE45D564-50CE-DA4F-89DD-50FC72A250F7}" name="TEMA 3E-3" dataDxfId="5"/>
-    <tableColumn id="25" xr3:uid="{84AA5875-DCCD-DF4B-8B28-6D92C876DED2}" name="ESTADO 3E" dataDxfId="4"/>
-    <tableColumn id="34" xr3:uid="{FA00F66E-CB06-E545-BD06-67E0A5E464B7}" name="PRACTICO" dataDxfId="3"/>
-    <tableColumn id="35" xr3:uid="{E5F86DDD-AB0D-C744-A246-1858A2347F20}" name="TALLERES" dataDxfId="2"/>
-    <tableColumn id="26" xr3:uid="{E1D0E942-C60E-094A-8858-8C730B93EAB9}" name="PARTICIPACION" dataDxfId="1"/>
-    <tableColumn id="28" xr3:uid="{810313C2-E5AF-AF41-82F7-A13FD739D191}" name="ESTADO" dataDxfId="0"/>
+    <tableColumn id="7" xr3:uid="{7C47C583-6454-7143-9A5D-CA0D6855FA55}" name="TEMA 1E-1" dataDxfId="45"/>
+    <tableColumn id="8" xr3:uid="{A89283B0-5A62-E944-B1EC-A79C9E8F0E9C}" name="TEMA 1E-2" dataDxfId="44"/>
+    <tableColumn id="9" xr3:uid="{0DC7A31D-F4E5-774F-89FF-1A4E80909842}" name="TEMA 1E-3" dataDxfId="43"/>
+    <tableColumn id="33" xr3:uid="{DA4A822E-2817-1244-BA2A-953AAFCACBAF}" name="TEMA 1E-4" dataDxfId="42"/>
+    <tableColumn id="10" xr3:uid="{7466F1D5-8437-AC4A-980C-A5AE857FF3CC}" name="ESTADO 1E" dataDxfId="41"/>
+    <tableColumn id="12" xr3:uid="{05A41B80-085C-D543-BD2B-67ED67375527}" name="FINAL" dataDxfId="40"/>
+    <tableColumn id="13" xr3:uid="{D9FF644A-C9F5-BE41-9011-B7F715418CA3}" name="EXAMEN 2E" dataDxfId="39"/>
+    <tableColumn id="14" xr3:uid="{B3ACF5E8-6AF9-D34C-B79B-F7EE5D15BEB7}" name="TEMA 2E-1.1" dataDxfId="38"/>
+    <tableColumn id="15" xr3:uid="{C76E2C0D-F2A6-3845-9675-078249A7096C}" name="TEMA 2E-1.2" dataDxfId="37"/>
+    <tableColumn id="16" xr3:uid="{DAAB7757-1235-DB49-8EA1-58E9C72DDF81}" name="TEMA 2E-2" dataDxfId="36"/>
+    <tableColumn id="18" xr3:uid="{BB97EC96-F05F-8F4D-989A-F6B50584BDC6}" name="ESTADO 2E" dataDxfId="35"/>
+    <tableColumn id="20" xr3:uid="{63AED625-1A4B-E447-8861-521ED4352977}" name="MEJORAMIENTO" dataDxfId="34"/>
+    <tableColumn id="21" xr3:uid="{4BDB3BC1-0532-944E-871E-8263817D8B94}" name="EXAMEN 3E" dataDxfId="33"/>
+    <tableColumn id="22" xr3:uid="{CA5D9BF3-B8F4-9F4D-B6BA-5F14BCD7D396}" name="TEMA 3E-1" dataDxfId="32"/>
+    <tableColumn id="23" xr3:uid="{C7E4476F-7BB9-3043-BB4F-0470EB216E0F}" name="TEMA 3E-2" dataDxfId="31"/>
+    <tableColumn id="24" xr3:uid="{CE45D564-50CE-DA4F-89DD-50FC72A250F7}" name="TEMA 3E-3" dataDxfId="30"/>
+    <tableColumn id="25" xr3:uid="{84AA5875-DCCD-DF4B-8B28-6D92C876DED2}" name="ESTADO 3E" dataDxfId="29"/>
+    <tableColumn id="34" xr3:uid="{FA00F66E-CB06-E545-BD06-67E0A5E464B7}" name="PRACTICO" dataDxfId="28"/>
+    <tableColumn id="35" xr3:uid="{E5F86DDD-AB0D-C744-A246-1858A2347F20}" name="TALLERES" dataDxfId="27"/>
+    <tableColumn id="26" xr3:uid="{E1D0E942-C60E-094A-8858-8C730B93EAB9}" name="PARTICIPACION" dataDxfId="26"/>
+    <tableColumn id="28" xr3:uid="{810313C2-E5AF-AF41-82F7-A13FD739D191}" name="ESTADO" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -2717,6 +4013,45 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{85DD1997-06F6-CD4D-BABC-95287E9C5EC3}" name="T_TPL_2025_26" displayName="T_TPL_2025_26" ref="A1:AD2">
+  <autoFilter ref="A1:AD2" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
+  <tableColumns count="30">
+    <tableColumn id="1" xr3:uid="{93BB635D-D0D8-CA4B-86AA-244400D9C949}" name="MATRICULA"/>
+    <tableColumn id="2" xr3:uid="{8DAE2FEF-E28F-7C4A-B32D-086263AC4CBA}" name="NOMBRE_ESTUDIANTE"/>
+    <tableColumn id="3" xr3:uid="{4F3167DE-853E-B545-AEEC-A3124484212F}" name="COD"/>
+    <tableColumn id="4" xr3:uid="{F8A064CB-DE2B-074D-8055-C12853D44BB5}" name="SIT"/>
+    <tableColumn id="5" xr3:uid="{32F14E0D-5450-F042-82F3-748067E0357B}" name="PARCIAL"/>
+    <tableColumn id="6" xr3:uid="{6F9A005A-F6C9-AA40-B2E2-403FDF402D76}" name="EXAMEN 1E"/>
+    <tableColumn id="7" xr3:uid="{B5FAF5AF-2BD3-134A-A05C-15833595D6ED}" name="TEMA 1E-1" dataDxfId="24"/>
+    <tableColumn id="8" xr3:uid="{641A1826-0CB6-CD47-A9A9-EE1F9AB61678}" name="TEMA 1E-2" dataDxfId="23"/>
+    <tableColumn id="9" xr3:uid="{6900A7FC-1B48-6D43-B15F-F759FC6A58B5}" name="TEMA 1E-3" dataDxfId="22"/>
+    <tableColumn id="10" xr3:uid="{BE1EB534-AE70-3D41-B5FC-8EA160A710F0}" name="ESTADO 1E" dataDxfId="21"/>
+    <tableColumn id="11" xr3:uid="{AB5852D8-396E-B44A-B10E-E8ED21918836}" name="REVISADO_X_ESTUDIANTE 1E" dataDxfId="20"/>
+    <tableColumn id="12" xr3:uid="{B4F4C4E7-983E-2A4B-8177-096E4D9751FB}" name="FINAL" dataDxfId="19"/>
+    <tableColumn id="13" xr3:uid="{2D382F08-D8DD-E841-9FA1-A76D48D7869F}" name="EXAMEN 2E" dataDxfId="18"/>
+    <tableColumn id="14" xr3:uid="{2635CA99-CAF7-C64C-A466-538937EEA017}" name="TEMA 2E-1" dataDxfId="17"/>
+    <tableColumn id="15" xr3:uid="{CF1D156E-5CC6-1041-8942-EE1E38B4424C}" name="TEMA 2E-2" dataDxfId="16"/>
+    <tableColumn id="16" xr3:uid="{206A20F8-E85D-0E42-AA0C-5A06809112CC}" name="TEMA 2E-3" dataDxfId="15"/>
+    <tableColumn id="18" xr3:uid="{F2E35C69-1424-B442-80A0-C7F970E6DE6F}" name="ESTADO 2E" dataDxfId="14"/>
+    <tableColumn id="19" xr3:uid="{8384044E-D86C-9741-B23D-4B4F932BF1DD}" name="REVISADO_X_ESTUDIANTE 2E" dataDxfId="13"/>
+    <tableColumn id="20" xr3:uid="{01EC63CD-D197-B046-AC3B-3A460005BF2D}" name="MEJORAMIENTO" dataDxfId="12"/>
+    <tableColumn id="21" xr3:uid="{17AF4E57-E297-7646-85C5-4F5AA92A0D56}" name="EXAMEN 3E" dataDxfId="11"/>
+    <tableColumn id="22" xr3:uid="{51CBBB73-47B3-7A4A-B358-CDCCAACCF6DA}" name="TEMA 3E-1" dataDxfId="10"/>
+    <tableColumn id="23" xr3:uid="{8BB0F72E-C34B-AB45-B3FF-533474415D24}" name="TEMA 3E-2" dataDxfId="9"/>
+    <tableColumn id="24" xr3:uid="{23931C47-B72C-A949-8C59-908E007876C5}" name="TEMA 3E-3" dataDxfId="8"/>
+    <tableColumn id="26" xr3:uid="{5AB06192-7A65-B945-9A9A-F1FE4812E597}" name="ESTADO 3E" dataDxfId="7"/>
+    <tableColumn id="27" xr3:uid="{28923F7D-D09F-DC4B-9BAC-E262E5F44E80}" name="REVISADO_X_ESTUDIANTE 3E" dataDxfId="6"/>
+    <tableColumn id="28" xr3:uid="{786398B8-A9FD-3042-8F02-D789F76BA1AF}" name="PRACTICO" dataDxfId="5"/>
+    <tableColumn id="29" xr3:uid="{EE8F2AA3-F0C2-1140-AC6F-C3E24181A02F}" name="TALLERES" dataDxfId="4"/>
+    <tableColumn id="30" xr3:uid="{A6B030D3-B2AB-4543-A8A4-91834706D632}" name="PARTICIPACION" dataDxfId="3"/>
+    <tableColumn id="31" xr3:uid="{9FACED0A-30CE-2C4B-8A81-5A5DC3B24A74}" name="TRABAJOS_EXTRA" dataDxfId="2"/>
+    <tableColumn id="32" xr3:uid="{AB51EDEE-9EF6-904C-8F5B-1847E5EBB6EA}" name="ESTADO" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="T_TPL_2025_1" displayName="T_TPL_2025_1" ref="A1:AF2">
   <autoFilter ref="A1:AF2" xr:uid="{00000000-0009-0000-0100-000007000000}"/>
   <tableColumns count="32">
@@ -2757,7 +4092,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="T_TPL_2025_2" displayName="T_TPL_2025_2" ref="A1:AE2">
   <autoFilter ref="A1:AE2" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
   <tableColumns count="31">
@@ -2792,6 +4127,48 @@
     <tableColumn id="29" xr3:uid="{00000000-0010-0000-0700-00001D000000}" name="PARTICIPACION"/>
     <tableColumn id="30" xr3:uid="{00000000-0010-0000-0700-00001E000000}" name="TRABAJOS_EXTRA"/>
     <tableColumn id="31" xr3:uid="{00000000-0010-0000-0700-00001F000000}" name="ESTADO"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{0CE27B1D-A37E-6940-A83B-BB5C74ECED31}" name="T_TPL_2025_2610" displayName="T_TPL_2025_2610" ref="A1:AG2">
+  <autoFilter ref="A1:AG2" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
+  <tableColumns count="33">
+    <tableColumn id="1" xr3:uid="{1AFDDF61-534F-2648-AE5C-E7E048E5ECFF}" name="MATRICULA"/>
+    <tableColumn id="2" xr3:uid="{2B829524-1F7F-4F44-A7DE-3A3E9C0215C3}" name="NOMBRE_ESTUDIANTE"/>
+    <tableColumn id="3" xr3:uid="{8C0E0425-BE9B-2046-9845-F9B7AF76C33F}" name="COD"/>
+    <tableColumn id="4" xr3:uid="{9BE32A72-4AF2-5144-876E-EB9453E4EC80}" name="SIT"/>
+    <tableColumn id="5" xr3:uid="{3AE820E8-BC9A-9E45-B1A7-EB92856E4779}" name="PARCIAL"/>
+    <tableColumn id="6" xr3:uid="{7CC6ABC5-F541-854E-9221-182E78E705F7}" name="EXAMEN 1E"/>
+    <tableColumn id="7" xr3:uid="{F38FB160-E4AE-5743-91D4-3D39359A0EF3}" name="TEMA 1E-1" dataDxfId="149"/>
+    <tableColumn id="8" xr3:uid="{5957C657-0BC3-B745-9DEF-2256CEA4F898}" name="TEMA 1E-2" dataDxfId="148"/>
+    <tableColumn id="9" xr3:uid="{2BBA5CEB-161C-C84B-91EC-0CFC52D8F566}" name="TEMA 1E-3" dataDxfId="147"/>
+    <tableColumn id="33" xr3:uid="{23F3E161-2759-8149-8AAA-BEFF97F622F4}" name="TEMA 1E-4" dataDxfId="0"/>
+    <tableColumn id="10" xr3:uid="{6E901AB2-C09C-0045-8631-0BAEB11DCD76}" name="ESTADO 1E" dataDxfId="146"/>
+    <tableColumn id="11" xr3:uid="{B392375C-E887-0D43-AE7F-0D621ED39533}" name="REVISADO_X_ESTUDIANTE" dataDxfId="145"/>
+    <tableColumn id="12" xr3:uid="{0A6E25AB-7FC6-5146-9C3D-F6C5AD77BD49}" name="FINAL" dataDxfId="144"/>
+    <tableColumn id="13" xr3:uid="{57AADA33-15DE-EE4B-B371-3EE210FD4887}" name="EXAMEN 2E" dataDxfId="143"/>
+    <tableColumn id="14" xr3:uid="{C2906A16-E333-974C-93DB-095E65371CBA}" name="TEMA 2E-1" dataDxfId="142"/>
+    <tableColumn id="15" xr3:uid="{A9C1CA64-00B5-5C4C-B635-98E0E06C85A6}" name="TEMA 2E-2" dataDxfId="141"/>
+    <tableColumn id="16" xr3:uid="{247D7B55-F8D0-5A42-9737-D4CB6EADC0A9}" name="TEMA 2E-3" dataDxfId="140"/>
+    <tableColumn id="17" xr3:uid="{D2C7A802-5044-1049-9EEA-4E3C86A18C36}" name="TEMA 2E-4" dataDxfId="139"/>
+    <tableColumn id="18" xr3:uid="{4C1DDBA6-9D9C-F94D-9915-D86EE9D3CD5D}" name="ESTADO 2E" dataDxfId="138"/>
+    <tableColumn id="19" xr3:uid="{F026DC93-CA76-8F4B-8166-2906AD67AA3E}" name="REVISADO_X_ESTUDIANTE 2E" dataDxfId="137"/>
+    <tableColumn id="20" xr3:uid="{4842DBD0-511E-6E4F-A4D6-C04752A3D2A7}" name="MEJORAMIENTO" dataDxfId="136"/>
+    <tableColumn id="21" xr3:uid="{001D1B2F-C76A-A84B-838B-222C47F8CD38}" name="EXAMEN 3E" dataDxfId="135"/>
+    <tableColumn id="22" xr3:uid="{B07EBC04-9CC3-7643-BFBD-79B0554ED698}" name="TEMA 3E-1" dataDxfId="134"/>
+    <tableColumn id="23" xr3:uid="{DEBFC8FB-A9DF-B34D-BCBD-F8B00507EF90}" name="TEMA 3E-2" dataDxfId="133"/>
+    <tableColumn id="24" xr3:uid="{1776AED2-06A0-8048-909B-1CF95FCBBB56}" name="TEMA 3E-3" dataDxfId="132"/>
+    <tableColumn id="25" xr3:uid="{71F38337-0240-014A-8043-DE94B937B9AA}" name="TEMA 3E-4" dataDxfId="131"/>
+    <tableColumn id="26" xr3:uid="{24B6298E-D8EC-3949-98DF-7CFF0E589ECD}" name="ESTADO 3E" dataDxfId="130"/>
+    <tableColumn id="27" xr3:uid="{58A3FC39-B516-8E4D-B396-3BEEADD8C646}" name="REVISADO_X_ESTUDIANTE 3E" dataDxfId="129"/>
+    <tableColumn id="28" xr3:uid="{014AD843-8A3D-6E41-A646-886672D931B8}" name="PRACTICO" dataDxfId="128"/>
+    <tableColumn id="29" xr3:uid="{0E193C08-CB64-1542-AD18-D9A1A11137D4}" name="TALLERES" dataDxfId="127"/>
+    <tableColumn id="30" xr3:uid="{AE07ACDC-C4FB-3D42-9C44-05730CC55322}" name="PARTICIPACION" dataDxfId="126"/>
+    <tableColumn id="31" xr3:uid="{A45C35FD-D0EB-9D4C-8C2A-8A566EA560C0}" name="TRABAJOS_EXTRA" dataDxfId="125"/>
+    <tableColumn id="32" xr3:uid="{8948F56A-40CF-9A40-B3A5-49837DE9E98C}" name="ESTADO" dataDxfId="124"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -4497,6 +5874,319 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4ECFA49-A5E1-8A48-A4B0-7DED1D2956AF}">
+  <dimension ref="A1:AD4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="19" customWidth="1"/>
+    <col min="3" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="28.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="26" customWidth="1"/>
+    <col min="13" max="17" width="12" customWidth="1"/>
+    <col min="18" max="18" width="26" customWidth="1"/>
+    <col min="19" max="19" width="14" customWidth="1"/>
+    <col min="20" max="23" width="12" customWidth="1"/>
+    <col min="24" max="24" width="26" customWidth="1"/>
+    <col min="25" max="26" width="12" customWidth="1"/>
+    <col min="27" max="27" width="15" customWidth="1"/>
+    <col min="28" max="28" width="16" customWidth="1"/>
+    <col min="29" max="29" width="13" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:30" ht="16" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q1" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="R1" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="S1" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="T1" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="U1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="V1" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="W1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="X1" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y1" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z1" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="AA1" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="AB1" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="AC1" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="AD1" s="10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:30" ht="16" x14ac:dyDescent="0.2">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="2">
+        <v>100</v>
+      </c>
+      <c r="F2" s="2">
+        <v>100</v>
+      </c>
+      <c r="G2" s="4">
+        <v>35</v>
+      </c>
+      <c r="H2" s="4">
+        <v>35</v>
+      </c>
+      <c r="I2" s="4">
+        <v>30</v>
+      </c>
+      <c r="J2" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="K2" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="L2" s="7">
+        <v>100</v>
+      </c>
+      <c r="M2" s="4">
+        <v>100</v>
+      </c>
+      <c r="N2" s="4">
+        <v>35</v>
+      </c>
+      <c r="O2" s="4">
+        <v>35</v>
+      </c>
+      <c r="P2" s="4">
+        <v>30</v>
+      </c>
+      <c r="Q2" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="R2" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="S2" s="12">
+        <v>100</v>
+      </c>
+      <c r="T2" s="6">
+        <v>100</v>
+      </c>
+      <c r="U2" s="6">
+        <v>40</v>
+      </c>
+      <c r="V2" s="6">
+        <v>40</v>
+      </c>
+      <c r="W2" s="6">
+        <v>20</v>
+      </c>
+      <c r="X2" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="Y2" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z2" s="13">
+        <v>100</v>
+      </c>
+      <c r="AA2" s="4">
+        <v>70</v>
+      </c>
+      <c r="AB2" s="4">
+        <v>30</v>
+      </c>
+      <c r="AC2" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="AD2" s="12" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" t="s">
+        <v>0</v>
+      </c>
+      <c r="F3" t="s">
+        <v>0</v>
+      </c>
+      <c r="G3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I3" t="s">
+        <v>55</v>
+      </c>
+      <c r="K3" t="s">
+        <v>0</v>
+      </c>
+      <c r="L3" t="s">
+        <v>0</v>
+      </c>
+      <c r="M3" t="s">
+        <v>0</v>
+      </c>
+      <c r="N3" t="s">
+        <v>58</v>
+      </c>
+      <c r="O3" t="s">
+        <v>60</v>
+      </c>
+      <c r="P3" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" t="s">
+        <v>0</v>
+      </c>
+      <c r="S3" t="s">
+        <v>0</v>
+      </c>
+      <c r="U3" t="s">
+        <v>57</v>
+      </c>
+      <c r="V3" t="s">
+        <v>54</v>
+      </c>
+      <c r="W3" t="s">
+        <v>59</v>
+      </c>
+      <c r="X3" t="s">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>0</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="G4" t="s">
+        <v>55</v>
+      </c>
+      <c r="H4" t="s">
+        <v>57</v>
+      </c>
+      <c r="I4" t="s">
+        <v>61</v>
+      </c>
+      <c r="N4" t="s">
+        <v>55</v>
+      </c>
+      <c r="O4" t="s">
+        <v>56</v>
+      </c>
+      <c r="U4" t="s">
+        <v>61</v>
+      </c>
+      <c r="V4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:AF4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -4835,7 +6525,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:AE4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -5163,4 +6853,338 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A43DDADD-8FDE-1D47-B404-E0A4DB3C25C9}">
+  <dimension ref="A1:AG4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="19" customWidth="1"/>
+    <col min="3" max="12" width="12" customWidth="1"/>
+    <col min="13" max="13" width="26" customWidth="1"/>
+    <col min="14" max="19" width="12" customWidth="1"/>
+    <col min="20" max="20" width="26" customWidth="1"/>
+    <col min="21" max="21" width="14" customWidth="1"/>
+    <col min="22" max="26" width="12" customWidth="1"/>
+    <col min="27" max="27" width="26" customWidth="1"/>
+    <col min="28" max="29" width="12" customWidth="1"/>
+    <col min="30" max="30" width="15" customWidth="1"/>
+    <col min="31" max="31" width="16" customWidth="1"/>
+    <col min="32" max="32" width="13" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:33" ht="16" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="J1" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="L1" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="S1" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="T1" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="U1" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="V1" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="W1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="X1" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="Y1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="Z1" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="AB1" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AC1" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="AD1" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="AE1" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="AF1" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="AG1" s="10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:33" ht="16" x14ac:dyDescent="0.2">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="2">
+        <v>100</v>
+      </c>
+      <c r="F2" s="2">
+        <v>100</v>
+      </c>
+      <c r="G2" s="4">
+        <v>25</v>
+      </c>
+      <c r="H2" s="4">
+        <v>25</v>
+      </c>
+      <c r="I2" s="4">
+        <v>25</v>
+      </c>
+      <c r="J2" s="4">
+        <v>25</v>
+      </c>
+      <c r="K2" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="L2" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="7">
+        <v>100</v>
+      </c>
+      <c r="N2" s="4">
+        <v>100</v>
+      </c>
+      <c r="O2" s="4">
+        <v>35</v>
+      </c>
+      <c r="P2" s="4">
+        <v>20</v>
+      </c>
+      <c r="Q2" s="4">
+        <v>45</v>
+      </c>
+      <c r="R2" s="4">
+        <v>0</v>
+      </c>
+      <c r="S2" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="T2" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="U2" s="12">
+        <v>100</v>
+      </c>
+      <c r="V2" s="6">
+        <v>100</v>
+      </c>
+      <c r="W2" s="6">
+        <v>20</v>
+      </c>
+      <c r="X2" s="6">
+        <v>20</v>
+      </c>
+      <c r="Y2" s="6">
+        <v>30</v>
+      </c>
+      <c r="Z2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA2" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="AB2" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="AC2" s="13">
+        <v>100</v>
+      </c>
+      <c r="AD2" s="4">
+        <v>70</v>
+      </c>
+      <c r="AE2" s="4">
+        <v>30</v>
+      </c>
+      <c r="AF2" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="AG2" s="12" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" t="s">
+        <v>0</v>
+      </c>
+      <c r="F3" t="s">
+        <v>0</v>
+      </c>
+      <c r="G3" t="s">
+        <v>67</v>
+      </c>
+      <c r="H3" t="s">
+        <v>55</v>
+      </c>
+      <c r="I3" t="s">
+        <v>56</v>
+      </c>
+      <c r="J3" t="s">
+        <v>61</v>
+      </c>
+      <c r="L3" t="s">
+        <v>0</v>
+      </c>
+      <c r="M3" t="s">
+        <v>0</v>
+      </c>
+      <c r="N3" t="s">
+        <v>0</v>
+      </c>
+      <c r="O3" t="s">
+        <v>60</v>
+      </c>
+      <c r="P3" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>59</v>
+      </c>
+      <c r="S3" t="s">
+        <v>0</v>
+      </c>
+      <c r="T3" t="s">
+        <v>0</v>
+      </c>
+      <c r="U3" t="s">
+        <v>0</v>
+      </c>
+      <c r="W3" t="s">
+        <v>60</v>
+      </c>
+      <c r="X3" t="s">
+        <v>58</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>59</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="H4" t="s">
+        <v>57</v>
+      </c>
+      <c r="I4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J4" t="s">
+        <v>57</v>
+      </c>
+      <c r="O4" t="s">
+        <v>56</v>
+      </c>
+      <c r="W4" t="s">
+        <v>55</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Agregando Ayudantías al dashboard
</commit_message>
<xml_diff>
--- a/metadata/metadata_estadisticas_FP.xlsx
+++ b/metadata/metadata_estadisticas_FP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/djurado/Projects/FP-History/metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{494A7E8B-6F43-FA42-A1E6-82F2C7BE253F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A712A520-EDF9-154F-BAFF-C102F8631C13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1640" yWindow="780" windowWidth="29400" windowHeight="18460" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7023,10 +7023,10 @@
         <v>100</v>
       </c>
       <c r="AC2" s="4">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="AD2" s="4">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="AE2" s="22" t="s">
         <v>13</v>

</xml_diff>